<commit_message>
fix: normalize NMC955 market to complete battery mass
The market declares one kilogram of battery but purchased only 0.72591 kg
of complete-pack manufacture. That fraction already represents the cell
content inside pack production, so applying it again at market level
understated manufacturing inputs.

Set the market manufacture input to 1 kg, preserve the internal cell
fraction and freight, and explain the boundary in workbook metadata and
the changelog. This fixes market normalization only; the separate anode
boundary and cell-performance issues remain for subsequent review.

Validation: a Brightway ExcelImporter regression failed on the original
0.72591 coefficient and passes after correction. Compare every workbook
cell and XLSX member: only B260 and documentation cell B252 changed;
all other values, formulas, styles and member contents are preserved.
Ruff, Black formatting and git diff --check pass.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-NMC955-LTO.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-NMC955-LTO.xlsx
@@ -5000,8 +5000,10 @@
       <c r="A252" t="s">
         <v>1</v>
       </c>
-      <c r="B252" t="s">
-        <v>290</v>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Modeled from the NMC622 inventory provided by Crenna et al., 2021., itself based on Dai et al., 2019. Market normalization correction: 1 kg of battery sold requires 1 kg of complete battery production. The 0.72591 kg cell fraction is already included in battery production and must not be applied again at market level.</t>
+        </is>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.2">
@@ -5088,7 +5090,7 @@
         <v>289</v>
       </c>
       <c r="B260">
-        <v>0.72591000000000006</v>
+        <v>1</v>
       </c>
       <c r="C260" t="s">
         <v>8</v>

</xml_diff>